<commit_message>
User Access Maintenance FRS v1.3 rebuilt with the new screenshots and screen texts; highlighted copy and workbooks rebuilt
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-11_User_Access_Maintenance/BIBS_UAT_BRD-11_Business_Unit_Walkthrough_Users_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-11_User_Access_Maintenance/BIBS_UAT_BRD-11_Business_Unit_Walkthrough_Users_v1.0.xlsx
@@ -867,7 +867,7 @@
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>BIBS UAT environment (address issued with the passwords). Password: Issued separately by the iorta TechNXT Project Team</t>
+          <t>BIBS UAT environment: https://uat.brokerverse.cloud. Password: Issued separately by the iorta TechNXT Project Team</t>
         </is>
       </c>
       <c r="D21" s="14" t="n">
@@ -923,7 +923,7 @@
     <row r="29">
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>Environment: BIBS UAT environment (address issued with the passwords). Passwords: Issued separately by the iorta TechNXT Project Team; no password is written in this workbook.</t>
+          <t>Environment: BIBS UAT environment: https://uat.brokerverse.cloud. Passwords: Issued separately by the iorta TechNXT Project Team; no password is written in this workbook.</t>
         </is>
       </c>
     </row>
@@ -1365,7 +1365,7 @@
     <row r="2">
       <c r="A2" s="23" t="inlineStr">
         <is>
-          <t>BIBS UAT environment (address issued with the passwords). Password: Issued separately by the iorta TechNXT Project Team</t>
+          <t>BIBS UAT environment: https://uat.brokerverse.cloud. Password: Issued separately by the iorta TechNXT Project Team</t>
         </is>
       </c>
     </row>

</xml_diff>